<commit_message>
feat(catalog): incorporar botella ergonomica de yogurt/jugo 500ml y actualizar planilla excel
- Descargar imagen de alta resolucion de Botella ergonomica tipo yogurt/jugo 500ml desde rclone
- Registrar producto en base de datos Supabase para ayme-pet con atributos y escalas de precios
- Actualizar plantilla_importacion_productos_ayme.xlsx en Google Drive con la nueva referencia
- Sincronizar catalogo en landing desacoplada de AYME
</commit_message>
<xml_diff>
--- a/plantilla_importacion_productos_ayme.xlsx
+++ b/plantilla_importacion_productos_ayme.xlsx
@@ -79,18 +79,48 @@
     <t>simple</t>
   </si>
   <si>
+    <t>AYME-YOG-500</t>
+  </si>
+  <si>
+    <t>Botella Ergonómica 500ml Tipo Yogurt o Jugo con Tapa Roscada</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>visible</t>
+  </si>
+  <si>
+    <t>Envase ergonómico de 500ml con cintura anatómica y tapa roscada estriada</t>
+  </si>
+  <si>
+    <t>Botella plástica PET/PEAD blanca de alta opacidad y protección contra luz UV. Diseño ergonómico de fácil agarre para yogurt, lácteos, jugos pasteurizados y néctares. Incluye tapa rosca con precinto de seguridad.</t>
+  </si>
+  <si>
+    <t>Envases para Alimentos, Contenedores Plásticos</t>
+  </si>
+  <si>
+    <t>yogurt, lacteos, jugos, ergonomica, 500ml</t>
+  </si>
+  <si>
+    <t>/assets/products/yogurt-500ml/1793204589665.jpg</t>
+  </si>
+  <si>
+    <t>Rosca 38mm / 28mm PCO</t>
+  </si>
+  <si>
+    <t>500 ml</t>
+  </si>
+  <si>
+    <t>28 g</t>
+  </si>
+  <si>
     <t>AYME-OSITO-250</t>
   </si>
   <si>
     <t>Envase / Botella Plástica Infantil Figura Osito 250ml con Tapa Roscada</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>visible</t>
-  </si>
-  <si>
     <t>Botella figura de osito 250ml con tapa rosca de alta hermeticidad</t>
   </si>
   <si>
@@ -145,9 +175,6 @@
     <t>28mm PCO / 38mm</t>
   </si>
   <si>
-    <t>500 ml</t>
-  </si>
-  <si>
     <t>45 g</t>
   </si>
   <si>
@@ -266,9 +293,6 @@
   </si>
   <si>
     <t>Boca de 63mm para fácil llenado y dosificación de salsas, frutos secos, polvos nutricionales y confitería.</t>
-  </si>
-  <si>
-    <t>Envases para Alimentos, Contenedores Plásticos</t>
   </si>
   <si>
     <t>frasco, boca ancha, 63mm, alimentos, confiteria</t>
@@ -518,13 +542,13 @@
         <v>23</v>
       </c>
       <c r="J2">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="K2">
-        <v>0.35</v>
+        <v>0.22</v>
       </c>
       <c r="L2">
-        <v>0.29</v>
+        <v>0.18</v>
       </c>
       <c r="M2" t="s">
         <v>27</v>
@@ -535,17 +559,14 @@
       <c r="O2" t="s">
         <v>29</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>30</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>31</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>32</v>
-      </c>
-      <c r="S2" t="s">
-        <v>33</v>
       </c>
       <c r="T2">
         <v>100</v>
@@ -556,10 +577,10 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
         <v>34</v>
-      </c>
-      <c r="C3" t="s">
-        <v>35</v>
       </c>
       <c r="D3" t="s">
         <v>23</v>
@@ -571,43 +592,43 @@
         <v>24</v>
       </c>
       <c r="G3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" t="s">
         <v>36</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3">
+        <v>15000</v>
+      </c>
+      <c r="K3">
+        <v>0.35</v>
+      </c>
+      <c r="L3">
+        <v>0.29</v>
+      </c>
+      <c r="M3" t="s">
         <v>37</v>
       </c>
-      <c r="I3" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3">
-        <v>10000</v>
-      </c>
-      <c r="K3">
-        <v>0.28</v>
-      </c>
-      <c r="L3">
-        <v>0.24</v>
-      </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>38</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>39</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>40</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>41</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>42</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>43</v>
-      </c>
-      <c r="S3" t="s">
-        <v>44</v>
       </c>
       <c r="T3">
         <v>100</v>
@@ -618,10 +639,10 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
         <v>45</v>
-      </c>
-      <c r="C4" t="s">
-        <v>46</v>
       </c>
       <c r="D4" t="s">
         <v>23</v>
@@ -633,25 +654,25 @@
         <v>24</v>
       </c>
       <c r="G4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" t="s">
         <v>47</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4">
+        <v>10000</v>
+      </c>
+      <c r="K4">
+        <v>0.28</v>
+      </c>
+      <c r="L4">
+        <v>0.24</v>
+      </c>
+      <c r="M4" t="s">
         <v>48</v>
-      </c>
-      <c r="I4" t="s">
-        <v>23</v>
-      </c>
-      <c r="J4">
-        <v>50000</v>
-      </c>
-      <c r="K4">
-        <v>0.18</v>
-      </c>
-      <c r="L4">
-        <v>0.15</v>
-      </c>
-      <c r="M4" t="s">
-        <v>27</v>
       </c>
       <c r="N4" t="s">
         <v>49</v>
@@ -659,14 +680,17 @@
       <c r="O4" t="s">
         <v>50</v>
       </c>
+      <c r="P4" t="s">
+        <v>51</v>
+      </c>
       <c r="Q4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R4" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="S4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="T4">
         <v>100</v>
@@ -677,10 +701,10 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
         <v>23</v>
@@ -692,37 +716,37 @@
         <v>24</v>
       </c>
       <c r="G5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I5" t="s">
         <v>23</v>
       </c>
       <c r="J5">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="K5">
-        <v>0.25</v>
+        <v>0.18</v>
       </c>
       <c r="L5">
-        <v>0.22</v>
+        <v>0.15</v>
       </c>
       <c r="M5" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="N5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="R5" t="s">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="S5" t="s">
         <v>61</v>
@@ -760,34 +784,34 @@
         <v>23</v>
       </c>
       <c r="J6">
-        <v>15000</v>
+        <v>30000</v>
       </c>
       <c r="K6">
-        <v>0.85</v>
+        <v>0.25</v>
       </c>
       <c r="L6">
-        <v>0.75</v>
+        <v>0.22</v>
       </c>
       <c r="M6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="N6" t="s">
         <v>66</v>
       </c>
       <c r="O6" t="s">
-        <v>40</v>
+        <v>67</v>
       </c>
       <c r="Q6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="R6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="S6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="T6">
-        <v>24</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -795,16 +819,16 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
       </c>
       <c r="E7" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="F7" t="s">
         <v>24</v>
@@ -819,34 +843,34 @@
         <v>23</v>
       </c>
       <c r="J7">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="K7">
-        <v>0.16</v>
+        <v>0.85</v>
       </c>
       <c r="L7">
-        <v>0.14</v>
+        <v>0.75</v>
       </c>
       <c r="M7" t="s">
+        <v>48</v>
+      </c>
+      <c r="N7" t="s">
         <v>75</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q7" t="s">
         <v>76</v>
       </c>
-      <c r="O7" t="s">
+      <c r="R7" t="s">
         <v>77</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="S7" t="s">
         <v>78</v>
       </c>
-      <c r="R7" t="s">
-        <v>32</v>
-      </c>
-      <c r="S7" t="s">
-        <v>79</v>
-      </c>
       <c r="T7">
-        <v>200</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -854,16 +878,16 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" t="s">
         <v>80</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" t="s">
         <v>81</v>
-      </c>
-      <c r="D8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" t="s">
-        <v>72</v>
       </c>
       <c r="F8" t="s">
         <v>24</v>
@@ -878,13 +902,13 @@
         <v>23</v>
       </c>
       <c r="J8">
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="K8">
-        <v>0.28</v>
+        <v>0.16</v>
       </c>
       <c r="L8">
-        <v>0.24</v>
+        <v>0.14</v>
       </c>
       <c r="M8" t="s">
         <v>84</v>
@@ -899,13 +923,13 @@
         <v>87</v>
       </c>
       <c r="R8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S8" t="s">
-        <v>61</v>
+        <v>88</v>
       </c>
       <c r="T8">
-        <v>120</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9">
@@ -913,25 +937,25 @@
         <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s">
         <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="F9" t="s">
         <v>24</v>
       </c>
       <c r="G9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I9" t="s">
         <v>23</v>
@@ -940,31 +964,31 @@
         <v>20000</v>
       </c>
       <c r="K9">
-        <v>0.32</v>
+        <v>0.28</v>
       </c>
       <c r="L9">
-        <v>0.28</v>
+        <v>0.24</v>
       </c>
       <c r="M9" t="s">
         <v>27</v>
       </c>
       <c r="N9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="O9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q9" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
       <c r="R9" t="s">
-        <v>94</v>
+        <v>31</v>
       </c>
       <c r="S9" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="T9">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10">
@@ -981,7 +1005,7 @@
         <v>23</v>
       </c>
       <c r="E10" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="F10" t="s">
         <v>24</v>
@@ -996,34 +1020,34 @@
         <v>23</v>
       </c>
       <c r="J10">
-        <v>100000</v>
+        <v>20000</v>
       </c>
       <c r="K10">
-        <v>0.1</v>
+        <v>0.32</v>
       </c>
       <c r="L10">
-        <v>0.085</v>
+        <v>0.28</v>
       </c>
       <c r="M10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" t="s">
         <v>100</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>101</v>
       </c>
-      <c r="O10" t="s">
+      <c r="Q10" t="s">
+        <v>68</v>
+      </c>
+      <c r="R10" t="s">
         <v>102</v>
       </c>
-      <c r="Q10" t="s">
-        <v>51</v>
-      </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>103</v>
       </c>
-      <c r="S10" t="s">
-        <v>104</v>
-      </c>
       <c r="T10">
-        <v>1000</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
@@ -1031,40 +1055,40 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" t="s">
         <v>105</v>
       </c>
-      <c r="C11" t="s">
-        <v>106</v>
-      </c>
       <c r="D11" t="s">
         <v>23</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="F11" t="s">
         <v>24</v>
       </c>
       <c r="G11" t="s">
+        <v>106</v>
+      </c>
+      <c r="H11" t="s">
         <v>107</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
+        <v>23</v>
+      </c>
+      <c r="J11">
+        <v>100000</v>
+      </c>
+      <c r="K11">
+        <v>0.1</v>
+      </c>
+      <c r="L11">
+        <v>0.085</v>
+      </c>
+      <c r="M11" t="s">
         <v>108</v>
-      </c>
-      <c r="I11" t="s">
-        <v>23</v>
-      </c>
-      <c r="J11">
-        <v>200000</v>
-      </c>
-      <c r="K11">
-        <v>0.04</v>
-      </c>
-      <c r="L11">
-        <v>0.032</v>
-      </c>
-      <c r="M11" t="s">
-        <v>100</v>
       </c>
       <c r="N11" t="s">
         <v>109</v>
@@ -1073,7 +1097,7 @@
         <v>110</v>
       </c>
       <c r="Q11" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="R11" t="s">
         <v>111</v>
@@ -1082,6 +1106,65 @@
         <v>112</v>
       </c>
       <c r="T11">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" t="s">
+        <v>115</v>
+      </c>
+      <c r="H12" t="s">
+        <v>116</v>
+      </c>
+      <c r="I12" t="s">
+        <v>23</v>
+      </c>
+      <c r="J12">
+        <v>200000</v>
+      </c>
+      <c r="K12">
+        <v>0.04</v>
+      </c>
+      <c r="L12">
+        <v>0.032</v>
+      </c>
+      <c r="M12" t="s">
+        <v>108</v>
+      </c>
+      <c r="N12" t="s">
+        <v>117</v>
+      </c>
+      <c r="O12" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>87</v>
+      </c>
+      <c r="R12" t="s">
+        <v>119</v>
+      </c>
+      <c r="S12" t="s">
+        <v>120</v>
+      </c>
+      <c r="T12">
         <v>5000</v>
       </c>
     </row>

</xml_diff>